<commit_message>
Fix Mini App: correct JSON field names, sync LIGA_OPTIONS, /start commands, template cleanup
</commit_message>
<xml_diff>
--- a/futbol_bot/apuestas_soccer.xlsx
+++ b/futbol_bot/apuestas_soccer.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z48"/>
+  <dimension ref="A1:Z55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1926,23 +1926,27 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>acertado</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>no_apostar</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>pendiente</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr"/>
+          <t>sin_datos</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>2 - 1.</t>
+        </is>
+      </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-06-06T22:21:03.724376</t>
+          <t>2026-06-06T23:02:41.374538</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -2110,17 +2114,25 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -2210,17 +2222,25 @@
           <t>Czechia</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -2310,17 +2330,25 @@
           <t>Bosnia-Herzegovina</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -2410,17 +2438,25 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -2510,17 +2546,25 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -2610,17 +2654,25 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -2710,17 +2762,25 @@
           <t>Scotland</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -2810,17 +2870,25 @@
           <t>Türkiye</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -2910,17 +2978,25 @@
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -3010,17 +3086,25 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -3110,17 +3194,25 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -3210,17 +3302,25 @@
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -3310,17 +3410,25 @@
           <t>Cape Verde</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -3410,17 +3518,25 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -3510,17 +3626,25 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -3610,17 +3734,25 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -3710,17 +3842,25 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -3810,17 +3950,25 @@
           <t>Norway</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -3910,17 +4058,25 @@
           <t>Algeria</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -4010,17 +4166,25 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -4110,17 +4274,25 @@
           <t>Congo DR</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -4210,17 +4382,25 @@
           <t>Croatia</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -4310,17 +4490,25 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -4410,17 +4598,25 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -4510,17 +4706,25 @@
           <t>South Africa</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -4610,17 +4814,25 @@
           <t>Bosnia-Herzegovina</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -4710,17 +4922,25 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -4810,17 +5030,25 @@
           <t>South Korea</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -4910,17 +5138,25 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>0</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -5010,17 +5246,25 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -5110,17 +5354,25 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -5210,17 +5462,25 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -5310,17 +5570,25 @@
           <t>Sweden</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -5410,17 +5678,25 @@
           <t>Ivory Coast</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -5510,17 +5786,25 @@
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>0</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -5584,6 +5868,804 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>4159559113272821804</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z49" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>4068069586459064018</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Málaga</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z50" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2606149404735617769</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Tigres UANL</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G51" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="O51" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="P51" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Over 4.5 Corners</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z51" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>14806177180014657630</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Aldosivi</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>AH0 - River Plate</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="O52" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="P52" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Over 4.5 Corners</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z52" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>10055280371506172102</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Sarmiento (Junín)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="O53" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="P53" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Over 4.5 Corners</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>10229698322051352208</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Godoy Cruz Antonio Tomba</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Mitre (Santiago del Estero)</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1517990362356477695</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AMISTOSOS_INT</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Boston River</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>NO_APOSTAR</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—  </t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>2026-06-07T06:00:01.466332</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="Z55" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>